<commit_message>
add project video link
</commit_message>
<xml_diff>
--- a/guru99_automation/target/test-classes/testdata/AccountId.xlsx
+++ b/guru99_automation/target/test-classes/testdata/AccountId.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
   <si>
     <t>AccountId</t>
   </si>
@@ -211,6 +211,18 @@
   </si>
   <si>
     <t>184446</t>
+  </si>
+  <si>
+    <t>184553</t>
+  </si>
+  <si>
+    <t>184554</t>
+  </si>
+  <si>
+    <t>184555</t>
+  </si>
+  <si>
+    <t>184556</t>
   </si>
 </sst>
 </file>
@@ -539,22 +551,22 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s" s="0">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="0" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="0" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s" s="0">
-        <v>61</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>